<commit_message>
new B7 graphite data
</commit_message>
<xml_diff>
--- a/GraphitePile/Results.xlsx
+++ b/GraphitePile/Results.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="28623"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29029"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\MCNP\b8\GraphitePile\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{05190C43-2820-4706-B1C7-2FEFF55B4899}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{76A4375A-C3C8-43E6-BDBB-4EC8DC26120F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="17496" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,29 +36,209 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="61" uniqueCount="59">
-  <si>
-    <t>Natural uranium</t>
-  </si>
-  <si>
-    <t>Density</t>
-  </si>
-  <si>
-    <t>EBC (ppm by mass)</t>
-  </si>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="80">
   <si>
     <t>Filename</t>
   </si>
   <si>
-    <t>Graphite</t>
-  </si>
-  <si>
     <t>k_eff</t>
   </si>
   <si>
     <t>unc</t>
   </si>
   <si>
+    <t>Pitch</t>
+  </si>
+  <si>
+    <t>o-seg-unit-Urho19_01-Uebc0-Grho1_70-Gebc0-pitch14.o</t>
+  </si>
+  <si>
+    <t>o-seg-unit-Urho19_01-Uebc0-Grho1_70-Gebc0-pitch15.o</t>
+  </si>
+  <si>
+    <t>o-seg-unit-Urho19_01-Uebc0-Grho1_70-Gebc0-pitch16.o</t>
+  </si>
+  <si>
+    <t>o-seg-unit-Urho19_01-Uebc0-Grho1_70-Gebc0-pitch17.o</t>
+  </si>
+  <si>
+    <t>o-seg-unit-Urho19_01-Uebc0-Grho1_70-Gebc0-pitch18.o</t>
+  </si>
+  <si>
+    <t>o-seg-unit-Urho19_01-Uebc0-Grho1_70-Gebc0-pitch19.o</t>
+  </si>
+  <si>
+    <t>o-seg-unit-Urho19_01-Uebc0-Grho1_70-Gebc0-pitch20.o</t>
+  </si>
+  <si>
+    <t>o-seg-unit-Urho19_01-Uebc0-Grho1_70-Gebc0-pitch21.o</t>
+  </si>
+  <si>
+    <t>o-seg-unit-Urho19_01-Uebc0-Grho1_70-Gebc0-pitch22.o</t>
+  </si>
+  <si>
+    <t>o-seg-unit-Urho19_01-Uebc0-Grho1_70-Gebc0-pitch23.o</t>
+  </si>
+  <si>
+    <t>o-seg-unit-Urho19_01-Uebc0-Grho1_70-Gebc0-pitch24.o</t>
+  </si>
+  <si>
+    <t>V_M/V_F</t>
+  </si>
+  <si>
+    <t>o-unit_cell-b8_u-agot_grph-pitch_14cm.o</t>
+  </si>
+  <si>
+    <t>o-unit_cell-b8_u-agot_grph-pitch_15cm.o</t>
+  </si>
+  <si>
+    <t>o-unit_cell-b8_u-agot_grph-pitch_16cm.o</t>
+  </si>
+  <si>
+    <t>o-unit_cell-b8_u-agot_grph-pitch_17cm.o</t>
+  </si>
+  <si>
+    <t>o-unit_cell-b8_u-agot_grph-pitch_18cm.o</t>
+  </si>
+  <si>
+    <t>o-unit_cell-b8_u-agot_grph-pitch_19cm.o</t>
+  </si>
+  <si>
+    <t>o-unit_cell-b8_u-agot_grph-pitch_20cm.o</t>
+  </si>
+  <si>
+    <t>o-unit_cell-b8_u-agot_grph-pitch_21cm.o</t>
+  </si>
+  <si>
+    <t>o-unit_cell-b8_u-agot_grph-pitch_22cm.o</t>
+  </si>
+  <si>
+    <t>o-unit_cell-b8_u-agot_grph-pitch_23cm.o</t>
+  </si>
+  <si>
+    <t>o-unit_cell-b8_u-agot_grph-pitch_24cm.o</t>
+  </si>
+  <si>
+    <t>o-unit_cell-b8_u-b7_grph-pitch_14cm.o</t>
+  </si>
+  <si>
+    <t>o-unit_cell-b8_u-b7_grph-pitch_15cm.o</t>
+  </si>
+  <si>
+    <t>o-unit_cell-b8_u-b7_grph-pitch_16cm.o</t>
+  </si>
+  <si>
+    <t>o-unit_cell-b8_u-b7_grph-pitch_17cm.o</t>
+  </si>
+  <si>
+    <t>o-unit_cell-b8_u-b7_grph-pitch_18cm.o</t>
+  </si>
+  <si>
+    <t>o-unit_cell-b8_u-b7_grph-pitch_19cm.o</t>
+  </si>
+  <si>
+    <t>o-unit_cell-b8_u-b7_grph-pitch_20cm.o</t>
+  </si>
+  <si>
+    <t>o-unit_cell-b8_u-b7_grph-pitch_21cm.o</t>
+  </si>
+  <si>
+    <t>o-unit_cell-b8_u-b7_grph-pitch_22cm.o</t>
+  </si>
+  <si>
+    <t>o-unit_cell-b8_u-b7_grph-pitch_23cm.o</t>
+  </si>
+  <si>
+    <t>o-unit_cell-b8_u-b7_grph-pitch_24cm.o</t>
+  </si>
+  <si>
+    <t>o-unit_cell-nominal_u-agot_grph-pitch_14cm.o</t>
+  </si>
+  <si>
+    <t>o-unit_cell-nominal_u-agot_grph-pitch_15cm.o</t>
+  </si>
+  <si>
+    <t>o-unit_cell-nominal_u-agot_grph-pitch_16cm.o</t>
+  </si>
+  <si>
+    <t>o-unit_cell-nominal_u-agot_grph-pitch_17cm.o</t>
+  </si>
+  <si>
+    <t>o-unit_cell-nominal_u-agot_grph-pitch_18cm.o</t>
+  </si>
+  <si>
+    <t>o-unit_cell-nominal_u-agot_grph-pitch_19cm.o</t>
+  </si>
+  <si>
+    <t>o-unit_cell-nominal_u-agot_grph-pitch_20cm.o</t>
+  </si>
+  <si>
+    <t>o-unit_cell-nominal_u-agot_grph-pitch_21cm.o</t>
+  </si>
+  <si>
+    <t>o-unit_cell-nominal_u-agot_grph-pitch_22cm.o</t>
+  </si>
+  <si>
+    <t>o-unit_cell-nominal_u-agot_grph-pitch_23cm.o</t>
+  </si>
+  <si>
+    <t>o-unit_cell-nominal_u-agot_grph-pitch_24cm.o</t>
+  </si>
+  <si>
+    <t>o-unit_cell-nominal_u-b7_grph-pitch_14cm.o</t>
+  </si>
+  <si>
+    <t>o-unit_cell-nominal_u-b7_grph-pitch_15cm.o</t>
+  </si>
+  <si>
+    <t>o-unit_cell-nominal_u-b7_grph-pitch_16cm.o</t>
+  </si>
+  <si>
+    <t>o-unit_cell-nominal_u-b7_grph-pitch_17cm.o</t>
+  </si>
+  <si>
+    <t>o-unit_cell-nominal_u-b7_grph-pitch_18cm.o</t>
+  </si>
+  <si>
+    <t>o-unit_cell-nominal_u-b7_grph-pitch_19cm.o</t>
+  </si>
+  <si>
+    <t>o-unit_cell-nominal_u-b7_grph-pitch_20cm.o</t>
+  </si>
+  <si>
+    <t>o-unit_cell-nominal_u-b7_grph-pitch_21cm.o</t>
+  </si>
+  <si>
+    <t>o-unit_cell-nominal_u-b7_grph-pitch_22cm.o</t>
+  </si>
+  <si>
+    <t>o-unit_cell-nominal_u-b7_grph-pitch_23cm.o</t>
+  </si>
+  <si>
+    <t>o-unit_cell-nominal_u-b7_grph-pitch_24cm.o</t>
+  </si>
+  <si>
+    <t>EBC (wppm)</t>
+  </si>
+  <si>
+    <t>U Density</t>
+  </si>
+  <si>
+    <t>Grph density</t>
+  </si>
+  <si>
+    <t>o-seg-unit-Urho19_01-Uebc0-Grho1_70-Gebc0-pitch25.o</t>
+  </si>
+  <si>
+    <t>o-seg-unit-Urho19_01-Uebc0-Grho1_70-Gebc0-pitch26.o</t>
+  </si>
+  <si>
+    <t>o-unit_cell-nominal_u-agot_grph-pitch_25cm.o</t>
+  </si>
+  <si>
+    <t>o-unit_cell-nominal_u-agot_grph-pitch_26cm.o</t>
+  </si>
+  <si>
     <t>o-seg-unit-Urho18_53-Uebc7_1-Grho1_70-Gebc6_6-pitch12.o</t>
   </si>
   <si>
@@ -86,139 +266,25 @@
     <t>o-seg-unit-Urho18_53-Uebc7_1-Grho1_70-Gebc6_6-pitch20.o</t>
   </si>
   <si>
-    <t>Pitch</t>
-  </si>
-  <si>
-    <t>o-seg-unit-Urho19_01-Uebc0-Grho1_70-Gebc0-pitch12.o</t>
-  </si>
-  <si>
-    <t>o-seg-unit-Urho19_01-Uebc0-Grho1_70-Gebc0-pitch13.o</t>
-  </si>
-  <si>
-    <t>o-seg-unit-Urho19_01-Uebc0-Grho1_70-Gebc0-pitch14.o</t>
-  </si>
-  <si>
-    <t>o-seg-unit-Urho19_01-Uebc0-Grho1_70-Gebc0-pitch15.o</t>
-  </si>
-  <si>
-    <t>o-seg-unit-Urho19_01-Uebc0-Grho1_70-Gebc0-pitch16.o</t>
-  </si>
-  <si>
-    <t>o-seg-unit-Urho19_01-Uebc0-Grho1_70-Gebc0-pitch17.o</t>
-  </si>
-  <si>
-    <t>o-seg-unit-Urho19_01-Uebc0-Grho1_70-Gebc0-pitch18.o</t>
-  </si>
-  <si>
-    <t>o-seg-unit-Urho19_01-Uebc0-Grho1_70-Gebc0-pitch19.o</t>
-  </si>
-  <si>
-    <t>o-seg-unit-Urho19_01-Uebc0-Grho1_70-Gebc0-pitch20.o</t>
-  </si>
-  <si>
-    <t>o-seg-unit-Urho19_01-Uebc0-Grho1_70-Gebc0-pitch21.o</t>
-  </si>
-  <si>
-    <t>o-seg-unit-Urho19_01-Uebc0-Grho1_70-Gebc0-pitch22.o</t>
-  </si>
-  <si>
-    <t>o-seg-unit-Urho19_01-Uebc0-Grho1_70-Gebc0-pitch23.o</t>
-  </si>
-  <si>
-    <t>o-seg-unit-Urho19_01-Uebc0-Grho1_70-Gebc0-pitch24.o</t>
-  </si>
-  <si>
-    <t>o-seg-unit-Urho18_53-Uebc7_1-Grho1_70-Gebc1_4-pitch12.o</t>
-  </si>
-  <si>
-    <t>o-seg-unit-Urho18_53-Uebc7_1-Grho1_70-Gebc1_4-pitch13.o</t>
-  </si>
-  <si>
-    <t>o-seg-unit-Urho18_53-Uebc7_1-Grho1_70-Gebc1_4-pitch14.o</t>
-  </si>
-  <si>
-    <t>o-seg-unit-Urho18_53-Uebc7_1-Grho1_70-Gebc1_4-pitch15.o</t>
-  </si>
-  <si>
-    <t>o-seg-unit-Urho18_53-Uebc7_1-Grho1_70-Gebc1_4-pitch16.o</t>
-  </si>
-  <si>
-    <t>V_M/V_F</t>
-  </si>
-  <si>
-    <t>o-seg-unit-Urho18_53-Uebc7_1-Grho1_70-Gebc1_4-pitch17.o</t>
-  </si>
-  <si>
-    <t>o-seg-unit-Urho18_53-Uebc7_1-Grho1_70-Gebc1_4-pitch18.o</t>
-  </si>
-  <si>
-    <t>o-seg-unit-Urho18_53-Uebc7_1-Grho1_70-Gebc1_4-pitch19.o</t>
-  </si>
-  <si>
-    <t>o-seg-unit-Urho18_53-Uebc7_1-Grho1_70-Gebc1_4-pitch20.o</t>
-  </si>
-  <si>
-    <t>o-seg-unit-Urho18_53-Uebc7_1-Grho1_70-Gebc1_4-pitch21.o</t>
-  </si>
-  <si>
-    <t>o-seg-unit-Urho18_53-Uebc7_1-Grho1_70-Gebc1_4-pitch22.o</t>
-  </si>
-  <si>
-    <t>o-seg-unit-Urho18_53-Uebc7_1-Grho1_70-Gebc1_4-pitch23.o</t>
-  </si>
-  <si>
-    <t>o-seg-unit-Urho18_53-Uebc7_1-Grho1_70-Gebc1_4-pitch24.o</t>
-  </si>
-  <si>
     <t>o-seg-unit-Urho18_53-Uebc7_1-Grho1_70-Gebc6_6-pitch21.o</t>
   </si>
   <si>
     <t>o-seg-unit-Urho18_53-Uebc7_1-Grho1_70-Gebc6_6-pitch22.o</t>
   </si>
   <si>
-    <t>o-seg-unit-Urho19_01-Uebc0-Grho1_70-Gebc6_6-pitch12.o</t>
-  </si>
-  <si>
-    <t>o-seg-unit-Urho19_01-Uebc0-Grho1_70-Gebc6_6-pitch13.o</t>
-  </si>
-  <si>
-    <t>o-seg-unit-Urho19_01-Uebc0-Grho1_70-Gebc6_6-pitch14.o</t>
-  </si>
-  <si>
-    <t>o-seg-unit-Urho19_01-Uebc0-Grho1_70-Gebc6_6-pitch15.o</t>
-  </si>
-  <si>
-    <t>o-seg-unit-Urho19_01-Uebc0-Grho1_70-Gebc6_6-pitch16.o</t>
-  </si>
-  <si>
-    <t>o-seg-unit-Urho19_01-Uebc0-Grho1_70-Gebc6_6-pitch17.o</t>
-  </si>
-  <si>
-    <t>o-seg-unit-Urho19_01-Uebc0-Grho1_70-Gebc6_6-pitch18.o</t>
-  </si>
-  <si>
-    <t>o-seg-unit-Urho19_01-Uebc0-Grho1_70-Gebc6_6-pitch19.o</t>
-  </si>
-  <si>
-    <t>o-seg-unit-Urho19_01-Uebc0-Grho1_70-Gebc6_6-pitch20.o</t>
-  </si>
-  <si>
-    <t>o-seg-unit-Urho19_01-Uebc0-Grho1_70-Gebc6_6-pitch21.o</t>
-  </si>
-  <si>
-    <t>o-seg-unit-Urho19_01-Uebc0-Grho1_70-Gebc6_6-pitch22.o</t>
-  </si>
-  <si>
-    <t>o-seg-unit-Urho19_01-Uebc0-Grho1_70-Gebc6_6-pitch23.o</t>
-  </si>
-  <si>
-    <t>o-seg-unit-Urho19_01-Uebc0-Grho1_70-Gebc6_6-pitch24.o</t>
+    <t>o-unit_cell-b8_u-agot_grph-pitch_25cm.o</t>
+  </si>
+  <si>
+    <t>o-unit_cell-b8_u-agot_grph-pitch_26cm.o</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="0.0"/>
+  </numFmts>
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -256,10 +322,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -268,9 +335,11 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFF38527"/>
+      <color rgb="FF41CD68"/>
+      <color rgb="FFF41859"/>
+      <color rgb="FFAD5DBC"/>
       <color rgb="FF009ADE"/>
-      <color rgb="FFF41859"/>
-      <color rgb="FF41CD68"/>
     </mruColors>
   </colors>
   <extLst>
@@ -307,11 +376,152 @@
         <c:ser>
           <c:idx val="0"/>
           <c:order val="0"/>
+          <c:spPr>
+            <a:ln w="19050" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="diamond"/>
+            <c:size val="6"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:srgbClr val="F41859"/>
+              </a:solidFill>
+              <a:ln w="12700">
+                <a:noFill/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="9525" cap="rnd">
+                <a:solidFill>
+                  <a:srgbClr val="F41859"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="poly"/>
+            <c:order val="4"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="0"/>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Sheet1!$F$2:$F$14</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="13"/>
+                <c:pt idx="0">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>21</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>22</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>23</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>24</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>26</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet1!$H$2:$H$14</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="13"/>
+                <c:pt idx="0">
+                  <c:v>0.96362999999999999</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1.0035099999999999</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1.03057</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1.04864</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1.05691</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1.0579000000000001</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1.05308</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1.0433600000000001</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1.0287299999999999</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1.0114099999999999</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.99102000000000001</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>0.96836</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>0.94374999999999998</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000000-F1AB-4E5B-B11A-2E6840E61FAC}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="1"/>
+          <c:order val="1"/>
           <c:tx>
-            <c:v>DegussaNU-SEG</c:v>
+            <c:v>"B8NU-B8grph"</c:v>
           </c:tx>
           <c:spPr>
-            <a:ln w="19050" cap="rnd">
+            <a:ln w="25400" cap="rnd">
               <a:noFill/>
               <a:round/>
             </a:ln>
@@ -324,7 +534,7 @@
               <a:solidFill>
                 <a:schemeClr val="tx1"/>
               </a:solidFill>
-              <a:ln w="12700">
+              <a:ln w="9525">
                 <a:noFill/>
               </a:ln>
               <a:effectLst/>
@@ -347,84 +557,84 @@
           </c:trendline>
           <c:xVal>
             <c:numRef>
-              <c:f>Sheet1!$F$3:$F$13</c:f>
+              <c:f>Sheet1!$F$16:$F$26</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="11"/>
                 <c:pt idx="0">
-                  <c:v>12</c:v>
+                  <c:v>14</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>13</c:v>
+                  <c:v>15</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>14</c:v>
+                  <c:v>16</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>15</c:v>
+                  <c:v>17</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>16</c:v>
+                  <c:v>18</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>17</c:v>
+                  <c:v>19</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>18</c:v>
+                  <c:v>20</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>19</c:v>
+                  <c:v>21</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>20</c:v>
+                  <c:v>22</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>21</c:v>
+                  <c:v>23</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>22</c:v>
+                  <c:v>24</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Sheet1!$H$3:$H$13</c:f>
+              <c:f>Sheet1!$H$16:$H$26</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="11"/>
                 <c:pt idx="0">
-                  <c:v>0.83423999999999998</c:v>
+                  <c:v>0.96059000000000005</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.89614000000000005</c:v>
+                  <c:v>0.99246999999999996</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.93979000000000001</c:v>
+                  <c:v>1.0120199999999999</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.96750000000000003</c:v>
+                  <c:v>1.0200499999999999</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.98211000000000004</c:v>
+                  <c:v>1.01922</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.98540000000000005</c:v>
+                  <c:v>1.01197</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.98006000000000004</c:v>
+                  <c:v>0.99856</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.96731</c:v>
+                  <c:v>0.97972999999999999</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.94891999999999999</c:v>
+                  <c:v>0.95721000000000001</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.92556000000000005</c:v>
+                  <c:v>0.93257000000000001</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.89922999999999997</c:v>
+                  <c:v>0.90500000000000003</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -432,16 +642,13 @@
           <c:smooth val="0"/>
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000000-F1AB-4E5B-B11A-2E6840E61FAC}"/>
+              <c16:uniqueId val="{00000002-F1AB-4E5B-B11A-2E6840E61FAC}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
         <c:ser>
-          <c:idx val="1"/>
-          <c:order val="1"/>
-          <c:tx>
-            <c:v>PureNu-PureG</c:v>
-          </c:tx>
+          <c:idx val="2"/>
+          <c:order val="2"/>
           <c:spPr>
             <a:ln w="25400" cap="rnd">
               <a:noFill/>
@@ -450,8 +657,8 @@
             <a:effectLst/>
           </c:spPr>
           <c:marker>
-            <c:symbol val="diamond"/>
-            <c:size val="7"/>
+            <c:symbol val="square"/>
+            <c:size val="5"/>
             <c:spPr>
               <a:solidFill>
                 <a:srgbClr val="41CD68"/>
@@ -479,240 +686,96 @@
           </c:trendline>
           <c:xVal>
             <c:numRef>
-              <c:f>Sheet1!$F$15:$F$27</c:f>
+              <c:f>Sheet1!$F$28:$F$40</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="13"/>
                 <c:pt idx="0">
-                  <c:v>12</c:v>
+                  <c:v>14</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>13</c:v>
+                  <c:v>15</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>14</c:v>
+                  <c:v>16</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>15</c:v>
+                  <c:v>17</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>16</c:v>
+                  <c:v>18</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>17</c:v>
+                  <c:v>19</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>18</c:v>
+                  <c:v>20</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>19</c:v>
+                  <c:v>21</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>20</c:v>
+                  <c:v>22</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>21</c:v>
+                  <c:v>23</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>22</c:v>
+                  <c:v>24</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>23</c:v>
+                  <c:v>25</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>24</c:v>
+                  <c:v>26</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Sheet1!$H$15:$H$27</c:f>
+              <c:f>Sheet1!$H$28:$H$40</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
                 <c:ptCount val="13"/>
                 <c:pt idx="0">
-                  <c:v>0.86136999999999997</c:v>
+                  <c:v>0.97521999999999998</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.93447999999999998</c:v>
+                  <c:v>1.0164299999999999</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.99070000000000003</c:v>
+                  <c:v>1.0458700000000001</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>1.0325800000000001</c:v>
+                  <c:v>1.0630500000000001</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>1.06219</c:v>
+                  <c:v>1.0724400000000001</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>1.0817099999999999</c:v>
+                  <c:v>1.0734300000000001</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>1.09256</c:v>
+                  <c:v>1.0687</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>1.09642</c:v>
+                  <c:v>1.0589999999999999</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>1.0943400000000001</c:v>
+                  <c:v>1.04487</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>1.08718</c:v>
+                  <c:v>1.0271600000000001</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>1.07606</c:v>
+                  <c:v>1.00644</c:v>
                 </c:pt>
                 <c:pt idx="11">
-                  <c:v>1.0610900000000001</c:v>
+                  <c:v>0.98375000000000001</c:v>
                 </c:pt>
                 <c:pt idx="12">
-                  <c:v>1.0434699999999999</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:yVal>
-          <c:smooth val="0"/>
-          <c:extLst>
-            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
-              <c16:uniqueId val="{00000002-F1AB-4E5B-B11A-2E6840E61FAC}"/>
-            </c:ext>
-          </c:extLst>
-        </c:ser>
-        <c:ser>
-          <c:idx val="2"/>
-          <c:order val="2"/>
-          <c:tx>
-            <c:v>DegussaNU-AGOT</c:v>
-          </c:tx>
-          <c:spPr>
-            <a:ln w="25400" cap="rnd">
-              <a:noFill/>
-              <a:round/>
-            </a:ln>
-            <a:effectLst/>
-          </c:spPr>
-          <c:marker>
-            <c:symbol val="square"/>
-            <c:size val="5"/>
-            <c:spPr>
-              <a:solidFill>
-                <a:srgbClr val="F41859"/>
-              </a:solidFill>
-              <a:ln w="9525">
-                <a:noFill/>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-          </c:marker>
-          <c:trendline>
-            <c:spPr>
-              <a:ln w="9525" cap="rnd">
-                <a:solidFill>
-                  <a:srgbClr val="F41859"/>
-                </a:solidFill>
-                <a:prstDash val="solid"/>
-              </a:ln>
-              <a:effectLst/>
-            </c:spPr>
-            <c:trendlineType val="poly"/>
-            <c:order val="4"/>
-            <c:dispRSqr val="0"/>
-            <c:dispEq val="0"/>
-          </c:trendline>
-          <c:xVal>
-            <c:numRef>
-              <c:f>Sheet1!$F$29:$F$41</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="13"/>
-                <c:pt idx="0">
-                  <c:v>12</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>13</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>14</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>15</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>16</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>17</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>18</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>19</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>20</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>21</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>22</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>23</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>24</c:v>
-                </c:pt>
-              </c:numCache>
-            </c:numRef>
-          </c:xVal>
-          <c:yVal>
-            <c:numRef>
-              <c:f>Sheet1!$H$29:$H$41</c:f>
-              <c:numCache>
-                <c:formatCode>General</c:formatCode>
-                <c:ptCount val="13"/>
-                <c:pt idx="0">
-                  <c:v>0.84845999999999999</c:v>
-                </c:pt>
-                <c:pt idx="1">
-                  <c:v>0.91712000000000005</c:v>
-                </c:pt>
-                <c:pt idx="2">
-                  <c:v>0.96872000000000003</c:v>
-                </c:pt>
-                <c:pt idx="3">
-                  <c:v>1.0056700000000001</c:v>
-                </c:pt>
-                <c:pt idx="4">
-                  <c:v>1.03034</c:v>
-                </c:pt>
-                <c:pt idx="5">
-                  <c:v>1.04437</c:v>
-                </c:pt>
-                <c:pt idx="6">
-                  <c:v>1.04986</c:v>
-                </c:pt>
-                <c:pt idx="7">
-                  <c:v>1.0482800000000001</c:v>
-                </c:pt>
-                <c:pt idx="8">
-                  <c:v>1.04074</c:v>
-                </c:pt>
-                <c:pt idx="9">
-                  <c:v>1.02807</c:v>
-                </c:pt>
-                <c:pt idx="10">
-                  <c:v>1.01156</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>0.99184000000000005</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>0.96913000000000005</c:v>
+                  <c:v>0.95835999999999999</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -727,9 +790,6 @@
         <c:ser>
           <c:idx val="3"/>
           <c:order val="3"/>
-          <c:tx>
-            <c:v>PureNU-SEG</c:v>
-          </c:tx>
           <c:spPr>
             <a:ln w="25400" cap="rnd">
               <a:noFill/>
@@ -767,47 +827,41 @@
           </c:trendline>
           <c:xVal>
             <c:numRef>
-              <c:f>Sheet1!$F$43:$F$55</c:f>
+              <c:f>Sheet1!$F$42:$F$52</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="13"/>
+                <c:ptCount val="11"/>
                 <c:pt idx="0">
-                  <c:v>12</c:v>
+                  <c:v>14</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>13</c:v>
+                  <c:v>15</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>14</c:v>
+                  <c:v>16</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>15</c:v>
+                  <c:v>17</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>16</c:v>
+                  <c:v>18</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>17</c:v>
+                  <c:v>19</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>18</c:v>
+                  <c:v>20</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>19</c:v>
+                  <c:v>21</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>20</c:v>
+                  <c:v>22</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>21</c:v>
+                  <c:v>23</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>22</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>23</c:v>
-                </c:pt>
-                <c:pt idx="12">
                   <c:v>24</c:v>
                 </c:pt>
               </c:numCache>
@@ -815,48 +869,42 @@
           </c:xVal>
           <c:yVal>
             <c:numRef>
-              <c:f>Sheet1!$H$43:$H$55</c:f>
+              <c:f>Sheet1!$H$42:$H$52</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="13"/>
+                <c:ptCount val="11"/>
                 <c:pt idx="0">
-                  <c:v>0.84230000000000005</c:v>
+                  <c:v>0.97228999999999999</c:v>
                 </c:pt>
                 <c:pt idx="1">
-                  <c:v>0.90561999999999998</c:v>
+                  <c:v>1.00552</c:v>
                 </c:pt>
                 <c:pt idx="2">
-                  <c:v>0.95065</c:v>
+                  <c:v>1.02549</c:v>
                 </c:pt>
                 <c:pt idx="3">
-                  <c:v>0.97985999999999995</c:v>
+                  <c:v>1.03454</c:v>
                 </c:pt>
                 <c:pt idx="4">
-                  <c:v>0.99507000000000001</c:v>
+                  <c:v>1.03451</c:v>
                 </c:pt>
                 <c:pt idx="5">
-                  <c:v>0.99902000000000002</c:v>
+                  <c:v>1.0269299999999999</c:v>
                 </c:pt>
                 <c:pt idx="6">
-                  <c:v>0.99387999999999999</c:v>
+                  <c:v>1.0133000000000001</c:v>
                 </c:pt>
                 <c:pt idx="7">
-                  <c:v>0.98128000000000004</c:v>
+                  <c:v>0.99485999999999997</c:v>
                 </c:pt>
                 <c:pt idx="8">
-                  <c:v>0.96287</c:v>
+                  <c:v>0.97267000000000003</c:v>
                 </c:pt>
                 <c:pt idx="9">
-                  <c:v>0.93959000000000004</c:v>
+                  <c:v>0.94721999999999995</c:v>
                 </c:pt>
                 <c:pt idx="10">
-                  <c:v>0.91279999999999994</c:v>
-                </c:pt>
-                <c:pt idx="11">
-                  <c:v>0.88341000000000003</c:v>
-                </c:pt>
-                <c:pt idx="12">
-                  <c:v>0.85238000000000003</c:v>
+                  <c:v>0.91939000000000004</c:v>
                 </c:pt>
               </c:numCache>
             </c:numRef>
@@ -865,6 +913,335 @@
           <c:extLst>
             <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
               <c16:uniqueId val="{00000004-A141-416A-AD9E-02BCA09A254F}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="4"/>
+          <c:order val="4"/>
+          <c:tx>
+            <c:v>1.03 line</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="9525" cap="rnd">
+              <a:solidFill>
+                <a:srgbClr val="FF0000"/>
+              </a:solidFill>
+              <a:prstDash val="lgDash"/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="circle"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:solidFill>
+                <a:schemeClr val="accent5"/>
+              </a:solidFill>
+              <a:ln w="9525">
+                <a:solidFill>
+                  <a:schemeClr val="accent5"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Sheet1!$K$24:$K$25</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="2"/>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet1!$L$24:$L$25</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="2"/>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000004-AA80-42DD-A67E-4F5A755185E1}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="5"/>
+          <c:order val="5"/>
+          <c:spPr>
+            <a:ln w="9525" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="x"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:srgbClr val="AD5DBC"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="9525" cap="rnd">
+                <a:solidFill>
+                  <a:srgbClr val="AD5DBC"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="poly"/>
+            <c:order val="4"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="0"/>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Sheet1!$F$54:$F$66</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="13"/>
+                <c:pt idx="0">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>21</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>22</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>23</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>24</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>25</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>26</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet1!$H$54:$H$66</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="13"/>
+                <c:pt idx="0">
+                  <c:v>0.99070000000000003</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>1.0325800000000001</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>1.06219</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>1.0817099999999999</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>1.09256</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>1.09642</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>1.0943400000000001</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>1.08718</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>1.07606</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>1.0610900000000001</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>1.0434699999999999</c:v>
+                </c:pt>
+                <c:pt idx="11">
+                  <c:v>1.02311</c:v>
+                </c:pt>
+                <c:pt idx="12">
+                  <c:v>1.00098</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000005-AA80-42DD-A67E-4F5A755185E1}"/>
+            </c:ext>
+          </c:extLst>
+        </c:ser>
+        <c:ser>
+          <c:idx val="6"/>
+          <c:order val="6"/>
+          <c:tx>
+            <c:v>B8NU-SEG</c:v>
+          </c:tx>
+          <c:spPr>
+            <a:ln w="25400" cap="rnd">
+              <a:noFill/>
+              <a:round/>
+            </a:ln>
+            <a:effectLst/>
+          </c:spPr>
+          <c:marker>
+            <c:symbol val="plus"/>
+            <c:size val="5"/>
+            <c:spPr>
+              <a:noFill/>
+              <a:ln w="19050">
+                <a:solidFill>
+                  <a:srgbClr val="F38527"/>
+                </a:solidFill>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+          </c:marker>
+          <c:trendline>
+            <c:spPr>
+              <a:ln w="9525" cap="rnd">
+                <a:solidFill>
+                  <a:srgbClr val="F38527"/>
+                </a:solidFill>
+                <a:prstDash val="solid"/>
+              </a:ln>
+              <a:effectLst/>
+            </c:spPr>
+            <c:trendlineType val="poly"/>
+            <c:order val="4"/>
+            <c:dispRSqr val="0"/>
+            <c:dispEq val="0"/>
+          </c:trendline>
+          <c:xVal>
+            <c:numRef>
+              <c:f>Sheet1!$F$68:$F$78</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="11"/>
+                <c:pt idx="0">
+                  <c:v>12</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>13</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>14</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>15</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>16</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>17</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>18</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>19</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>20</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>21</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>22</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:xVal>
+          <c:yVal>
+            <c:numRef>
+              <c:f>Sheet1!$H$68:$H$78</c:f>
+              <c:numCache>
+                <c:formatCode>General</c:formatCode>
+                <c:ptCount val="11"/>
+                <c:pt idx="0">
+                  <c:v>0.83423999999999998</c:v>
+                </c:pt>
+                <c:pt idx="1">
+                  <c:v>0.89614000000000005</c:v>
+                </c:pt>
+                <c:pt idx="2">
+                  <c:v>0.93979000000000001</c:v>
+                </c:pt>
+                <c:pt idx="3">
+                  <c:v>0.96750000000000003</c:v>
+                </c:pt>
+                <c:pt idx="4">
+                  <c:v>0.98211000000000004</c:v>
+                </c:pt>
+                <c:pt idx="5">
+                  <c:v>0.98540000000000005</c:v>
+                </c:pt>
+                <c:pt idx="6">
+                  <c:v>0.98006000000000004</c:v>
+                </c:pt>
+                <c:pt idx="7">
+                  <c:v>0.96731</c:v>
+                </c:pt>
+                <c:pt idx="8">
+                  <c:v>0.94891999999999999</c:v>
+                </c:pt>
+                <c:pt idx="9">
+                  <c:v>0.92556000000000005</c:v>
+                </c:pt>
+                <c:pt idx="10">
+                  <c:v>0.89922999999999997</c:v>
+                </c:pt>
+              </c:numCache>
+            </c:numRef>
+          </c:yVal>
+          <c:smooth val="0"/>
+          <c:extLst>
+            <c:ext xmlns:c16="http://schemas.microsoft.com/office/drawing/2014/chart" uri="{C3380CC4-5D6E-409C-BE32-E72D297353CC}">
+              <c16:uniqueId val="{00000005-9E7F-47C2-8670-96B1A3970865}"/>
             </c:ext>
           </c:extLst>
         </c:ser>
@@ -883,7 +1260,7 @@
         <c:axId val="899541711"/>
         <c:scaling>
           <c:orientation val="minMax"/>
-          <c:max val="24"/>
+          <c:max val="26"/>
           <c:min val="14"/>
         </c:scaling>
         <c:delete val="0"/>
@@ -990,8 +1367,8 @@
         <c:axId val="899546031"/>
         <c:scaling>
           <c:orientation val="minMax"/>
-          <c:max val="1.1200000000000001"/>
-          <c:min val="0.92"/>
+          <c:max val="1.1100000000000001"/>
+          <c:min val="0.95000000000000007"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
@@ -1091,7 +1468,7 @@
         <c:crosses val="autoZero"/>
         <c:crossBetween val="midCat"/>
         <c:majorUnit val="2.0000000000000004E-2"/>
-        <c:minorUnit val="2.0000000000000004E-2"/>
+        <c:minorUnit val="1.0000000000000002E-2"/>
       </c:valAx>
       <c:spPr>
         <a:noFill/>
@@ -1105,6 +1482,7 @@
     </c:plotArea>
     <c:plotVisOnly val="1"/>
     <c:dispBlanksAs val="gap"/>
+    <c:showDLblsOverMax val="0"/>
     <c:extLst>
       <c:ext xmlns:c16r3="http://schemas.microsoft.com/office/drawing/2017/03/chart" uri="{56B9EC1D-385E-4148-901F-78D8002777C0}">
         <c16r3:dataDisplayOptions16>
@@ -1112,7 +1490,6 @@
         </c16r3:dataDisplayOptions16>
       </c:ext>
     </c:extLst>
-    <c:showDLblsOverMax val="0"/>
   </c:chart>
   <c:spPr>
     <a:noFill/>
@@ -1700,16 +2077,16 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>9</xdr:col>
-      <xdr:colOff>83820</xdr:colOff>
-      <xdr:row>5</xdr:row>
-      <xdr:rowOff>30480</xdr:rowOff>
+      <xdr:col>8</xdr:col>
+      <xdr:colOff>351834</xdr:colOff>
+      <xdr:row>1</xdr:row>
+      <xdr:rowOff>19970</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>15</xdr:col>
-      <xdr:colOff>83820</xdr:colOff>
-      <xdr:row>20</xdr:row>
-      <xdr:rowOff>139504</xdr:rowOff>
+      <xdr:col>14</xdr:col>
+      <xdr:colOff>351834</xdr:colOff>
+      <xdr:row>16</xdr:row>
+      <xdr:rowOff>4203</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
       <xdr:nvGraphicFramePr>
@@ -2000,7 +2377,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I55"/>
+  <dimension ref="A1:I78"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="53.5546875" customWidth="1"/>
@@ -2011,1400 +2388,1990 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
       <c r="B1" s="1" t="s">
-        <v>0</v>
+        <v>61</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>60</v>
       </c>
       <c r="D1" s="1" t="s">
-        <v>4</v>
+        <v>62</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>2</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A2" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="B2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C2" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D2" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="E2" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="F2" s="1" t="s">
+      <c r="A2" t="s">
         <v>16</v>
       </c>
-      <c r="G2" s="1" t="s">
-        <v>35</v>
-      </c>
-      <c r="H2" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>6</v>
+      <c r="B2">
+        <v>18.5349</v>
+      </c>
+      <c r="C2" s="3">
+        <v>7</v>
+      </c>
+      <c r="D2" s="2">
+        <v>1.6</v>
+      </c>
+      <c r="E2">
+        <v>1.4</v>
+      </c>
+      <c r="F2">
+        <v>14</v>
+      </c>
+      <c r="G2" s="2">
+        <f>((F2^3)-(5^3))/(5^3)</f>
+        <v>20.952000000000002</v>
+      </c>
+      <c r="H2">
+        <v>0.96362999999999999</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
+        <v>17</v>
+      </c>
+      <c r="B3">
+        <v>18.5349</v>
+      </c>
+      <c r="C3" s="3">
         <v>7</v>
       </c>
-      <c r="B3">
-        <v>18.53</v>
-      </c>
-      <c r="C3">
-        <v>7.1</v>
-      </c>
       <c r="D3" s="2">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="E3">
-        <v>6.6</v>
+        <v>1.4</v>
       </c>
       <c r="F3">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="G3" s="2">
-        <f>((F3^3)-(5^3))/(5^3)</f>
-        <v>12.824</v>
+        <f t="shared" ref="G3:G64" si="0">((F3^3)-(5^3))/(5^3)</f>
+        <v>26</v>
       </c>
       <c r="H3">
-        <v>0.83423999999999998</v>
+        <v>1.0035099999999999</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="B4">
-        <v>18.53</v>
-      </c>
-      <c r="C4">
-        <v>7.1</v>
+        <v>18.5349</v>
+      </c>
+      <c r="C4" s="3">
+        <v>7</v>
       </c>
       <c r="D4" s="2">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="E4">
-        <v>6.6</v>
+        <v>1.4</v>
       </c>
       <c r="F4">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="G4" s="2">
-        <f t="shared" ref="G4:G55" si="0">((F4^3)-(5^3))/(5^3)</f>
-        <v>16.576000000000001</v>
+        <f t="shared" si="0"/>
+        <v>31.768000000000001</v>
       </c>
       <c r="H4">
-        <v>0.89614000000000005</v>
+        <v>1.03057</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
-        <v>9</v>
+        <v>19</v>
       </c>
       <c r="B5">
-        <v>18.53</v>
-      </c>
-      <c r="C5">
-        <v>7.1</v>
+        <v>18.5349</v>
+      </c>
+      <c r="C5" s="3">
+        <v>7</v>
       </c>
       <c r="D5" s="2">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="E5">
-        <v>6.6</v>
+        <v>1.4</v>
       </c>
       <c r="F5">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="G5" s="2">
         <f t="shared" si="0"/>
-        <v>20.952000000000002</v>
+        <v>38.304000000000002</v>
       </c>
       <c r="H5">
-        <v>0.93979000000000001</v>
+        <v>1.04864</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
-        <v>10</v>
+        <v>20</v>
       </c>
       <c r="B6">
-        <v>18.53</v>
-      </c>
-      <c r="C6">
-        <v>7.1</v>
+        <v>18.5349</v>
+      </c>
+      <c r="C6" s="3">
+        <v>7</v>
       </c>
       <c r="D6" s="2">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="E6">
-        <v>6.6</v>
+        <v>1.4</v>
       </c>
       <c r="F6">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="G6" s="2">
         <f t="shared" si="0"/>
-        <v>26</v>
+        <v>45.655999999999999</v>
       </c>
       <c r="H6">
-        <v>0.96750000000000003</v>
+        <v>1.05691</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
-        <v>11</v>
+        <v>21</v>
       </c>
       <c r="B7">
-        <v>18.53</v>
-      </c>
-      <c r="C7">
-        <v>7.1</v>
+        <v>18.5349</v>
+      </c>
+      <c r="C7" s="3">
+        <v>7</v>
       </c>
       <c r="D7" s="2">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="E7">
-        <v>6.6</v>
+        <v>1.4</v>
       </c>
       <c r="F7">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="G7" s="2">
         <f t="shared" si="0"/>
-        <v>31.768000000000001</v>
+        <v>53.872</v>
       </c>
       <c r="H7">
-        <v>0.98211000000000004</v>
+        <v>1.0579000000000001</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
-        <v>12</v>
+        <v>22</v>
       </c>
       <c r="B8">
-        <v>18.53</v>
-      </c>
-      <c r="C8">
-        <v>7.1</v>
+        <v>18.5349</v>
+      </c>
+      <c r="C8" s="3">
+        <v>7</v>
       </c>
       <c r="D8" s="2">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="E8">
-        <v>6.6</v>
+        <v>1.4</v>
       </c>
       <c r="F8">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="G8" s="2">
         <f t="shared" si="0"/>
-        <v>38.304000000000002</v>
+        <v>63</v>
       </c>
       <c r="H8">
-        <v>0.98540000000000005</v>
+        <v>1.05308</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
-        <v>13</v>
+        <v>23</v>
       </c>
       <c r="B9">
-        <v>18.53</v>
-      </c>
-      <c r="C9">
-        <v>7.1</v>
+        <v>18.5349</v>
+      </c>
+      <c r="C9" s="3">
+        <v>7</v>
       </c>
       <c r="D9" s="2">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="E9">
-        <v>6.6</v>
+        <v>1.4</v>
       </c>
       <c r="F9">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="G9" s="2">
         <f t="shared" si="0"/>
-        <v>45.655999999999999</v>
+        <v>73.087999999999994</v>
       </c>
       <c r="H9">
-        <v>0.98006000000000004</v>
+        <v>1.0433600000000001</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
-        <v>14</v>
+        <v>24</v>
       </c>
       <c r="B10">
-        <v>18.53</v>
-      </c>
-      <c r="C10">
-        <v>7.1</v>
+        <v>18.5349</v>
+      </c>
+      <c r="C10" s="3">
+        <v>7</v>
       </c>
       <c r="D10" s="2">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="E10">
-        <v>6.6</v>
+        <v>1.4</v>
       </c>
       <c r="F10">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="G10" s="2">
         <f t="shared" si="0"/>
-        <v>53.872</v>
+        <v>84.183999999999997</v>
       </c>
       <c r="H10">
-        <v>0.96731</v>
+        <v>1.0287299999999999</v>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
-        <v>15</v>
+        <v>25</v>
       </c>
       <c r="B11">
-        <v>18.53</v>
-      </c>
-      <c r="C11">
-        <v>7.1</v>
+        <v>18.5349</v>
+      </c>
+      <c r="C11" s="3">
+        <v>7</v>
       </c>
       <c r="D11" s="2">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="E11">
-        <v>6.6</v>
+        <v>1.4</v>
       </c>
       <c r="F11">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="G11" s="2">
         <f t="shared" si="0"/>
-        <v>63</v>
+        <v>96.335999999999999</v>
       </c>
       <c r="H11">
-        <v>0.94891999999999999</v>
+        <v>1.0114099999999999</v>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
-        <v>44</v>
+        <v>26</v>
       </c>
       <c r="B12">
-        <v>18.53</v>
-      </c>
-      <c r="C12">
-        <v>7.1</v>
+        <v>18.5349</v>
+      </c>
+      <c r="C12" s="3">
+        <v>7</v>
       </c>
       <c r="D12" s="2">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="E12">
-        <v>6.6</v>
+        <v>1.4</v>
       </c>
       <c r="F12">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="G12" s="2">
         <f t="shared" si="0"/>
-        <v>73.087999999999994</v>
+        <v>109.592</v>
       </c>
       <c r="H12">
-        <v>0.92556000000000005</v>
+        <v>0.99102000000000001</v>
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
-        <v>45</v>
+        <v>78</v>
       </c>
       <c r="B13">
-        <v>18.53</v>
-      </c>
-      <c r="C13">
-        <v>7.1</v>
+        <v>18.5349</v>
+      </c>
+      <c r="C13" s="3">
+        <v>7</v>
       </c>
       <c r="D13" s="2">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="E13">
-        <v>6.6</v>
+        <v>1.4</v>
       </c>
       <c r="F13">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="G13" s="2">
-        <f t="shared" si="0"/>
-        <v>84.183999999999997</v>
+        <f>((F13^3)-(5^3))/(5^3)</f>
+        <v>124</v>
       </c>
       <c r="H13">
-        <v>0.89922999999999997</v>
+        <v>0.96836</v>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="G14" s="2"/>
+      <c r="A14" t="s">
+        <v>79</v>
+      </c>
+      <c r="B14">
+        <v>18.5349</v>
+      </c>
+      <c r="C14" s="3">
+        <v>7</v>
+      </c>
+      <c r="D14" s="2">
+        <v>1.6</v>
+      </c>
+      <c r="E14">
+        <v>1.4</v>
+      </c>
+      <c r="F14">
+        <v>26</v>
+      </c>
+      <c r="G14" s="2">
+        <f t="shared" ref="G14" si="1">((F14^3)-(5^3))/(5^3)</f>
+        <v>139.608</v>
+      </c>
+      <c r="H14">
+        <v>0.94374999999999998</v>
+      </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="A15" t="s">
-        <v>17</v>
-      </c>
-      <c r="B15">
-        <v>19.010000000000002</v>
-      </c>
-      <c r="C15">
-        <v>0</v>
-      </c>
-      <c r="D15" s="2">
-        <v>1.7</v>
-      </c>
-      <c r="E15">
-        <v>0</v>
-      </c>
-      <c r="F15">
-        <v>12</v>
-      </c>
-      <c r="G15" s="2">
-        <f t="shared" si="0"/>
-        <v>12.824</v>
-      </c>
-      <c r="H15">
-        <v>0.86136999999999997</v>
-      </c>
+      <c r="G15" s="2"/>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.3">
       <c r="A16" t="s">
-        <v>18</v>
+        <v>27</v>
       </c>
       <c r="B16">
-        <v>19.010000000000002</v>
-      </c>
-      <c r="C16">
-        <v>0</v>
+        <v>18.5349</v>
+      </c>
+      <c r="C16" s="3">
+        <v>7</v>
       </c>
       <c r="D16" s="2">
         <v>1.7</v>
       </c>
       <c r="E16">
-        <v>0</v>
+        <v>3.4</v>
       </c>
       <c r="F16">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="G16" s="2">
         <f t="shared" si="0"/>
-        <v>16.576000000000001</v>
+        <v>20.952000000000002</v>
       </c>
       <c r="H16">
-        <v>0.93447999999999998</v>
+        <v>0.96059000000000005</v>
       </c>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A17" t="s">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="B17">
-        <v>19.010000000000002</v>
-      </c>
-      <c r="C17">
-        <v>0</v>
+        <v>18.5349</v>
+      </c>
+      <c r="C17" s="3">
+        <v>7</v>
       </c>
       <c r="D17" s="2">
         <v>1.7</v>
       </c>
       <c r="E17">
-        <v>0</v>
+        <v>3.4</v>
       </c>
       <c r="F17">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="G17" s="2">
         <f t="shared" si="0"/>
-        <v>20.952000000000002</v>
+        <v>26</v>
       </c>
       <c r="H17">
-        <v>0.99070000000000003</v>
+        <v>0.99246999999999996</v>
       </c>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A18" t="s">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="B18">
-        <v>19.010000000000002</v>
-      </c>
-      <c r="C18">
-        <v>0</v>
+        <v>18.5349</v>
+      </c>
+      <c r="C18" s="3">
+        <v>7</v>
       </c>
       <c r="D18" s="2">
         <v>1.7</v>
       </c>
       <c r="E18">
-        <v>0</v>
+        <v>3.4</v>
       </c>
       <c r="F18">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="G18" s="2">
         <f t="shared" si="0"/>
-        <v>26</v>
+        <v>31.768000000000001</v>
       </c>
       <c r="H18">
-        <v>1.0325800000000001</v>
+        <v>1.0120199999999999</v>
       </c>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" t="s">
-        <v>21</v>
+        <v>30</v>
       </c>
       <c r="B19">
-        <v>19.010000000000002</v>
-      </c>
-      <c r="C19">
-        <v>0</v>
+        <v>18.5349</v>
+      </c>
+      <c r="C19" s="3">
+        <v>7</v>
       </c>
       <c r="D19" s="2">
         <v>1.7</v>
       </c>
       <c r="E19">
-        <v>0</v>
+        <v>3.4</v>
       </c>
       <c r="F19">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="G19" s="2">
         <f t="shared" si="0"/>
-        <v>31.768000000000001</v>
+        <v>38.304000000000002</v>
       </c>
       <c r="H19">
-        <v>1.06219</v>
+        <v>1.0200499999999999</v>
       </c>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A20" t="s">
-        <v>22</v>
+        <v>31</v>
       </c>
       <c r="B20">
-        <v>19.010000000000002</v>
-      </c>
-      <c r="C20">
-        <v>0</v>
+        <v>18.5349</v>
+      </c>
+      <c r="C20" s="3">
+        <v>7</v>
       </c>
       <c r="D20" s="2">
         <v>1.7</v>
       </c>
       <c r="E20">
-        <v>0</v>
+        <v>3.4</v>
       </c>
       <c r="F20">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="G20" s="2">
         <f t="shared" si="0"/>
-        <v>38.304000000000002</v>
+        <v>45.655999999999999</v>
       </c>
       <c r="H20">
-        <v>1.0817099999999999</v>
+        <v>1.01922</v>
       </c>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A21" t="s">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="B21">
-        <v>19.010000000000002</v>
-      </c>
-      <c r="C21">
-        <v>0</v>
+        <v>18.5349</v>
+      </c>
+      <c r="C21" s="3">
+        <v>7</v>
       </c>
       <c r="D21" s="2">
         <v>1.7</v>
       </c>
       <c r="E21">
-        <v>0</v>
+        <v>3.4</v>
       </c>
       <c r="F21">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="G21" s="2">
         <f t="shared" si="0"/>
-        <v>45.655999999999999</v>
+        <v>53.872</v>
       </c>
       <c r="H21">
-        <v>1.09256</v>
+        <v>1.01197</v>
       </c>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A22" t="s">
-        <v>24</v>
+        <v>33</v>
       </c>
       <c r="B22">
-        <v>19.010000000000002</v>
-      </c>
-      <c r="C22">
-        <v>0</v>
+        <v>18.5349</v>
+      </c>
+      <c r="C22" s="3">
+        <v>7</v>
       </c>
       <c r="D22" s="2">
         <v>1.7</v>
       </c>
       <c r="E22">
-        <v>0</v>
+        <v>3.4</v>
       </c>
       <c r="F22">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="G22" s="2">
         <f t="shared" si="0"/>
-        <v>53.872</v>
+        <v>63</v>
       </c>
       <c r="H22">
-        <v>1.09642</v>
+        <v>0.99856</v>
       </c>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A23" t="s">
-        <v>25</v>
+        <v>34</v>
       </c>
       <c r="B23">
-        <v>19.010000000000002</v>
-      </c>
-      <c r="C23">
-        <v>0</v>
+        <v>18.5349</v>
+      </c>
+      <c r="C23" s="3">
+        <v>7</v>
       </c>
       <c r="D23" s="2">
         <v>1.7</v>
       </c>
       <c r="E23">
-        <v>0</v>
+        <v>3.4</v>
       </c>
       <c r="F23">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G23" s="2">
         <f t="shared" si="0"/>
-        <v>63</v>
+        <v>73.087999999999994</v>
       </c>
       <c r="H23">
-        <v>1.0943400000000001</v>
+        <v>0.97972999999999999</v>
       </c>
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A24" t="s">
-        <v>26</v>
+        <v>35</v>
       </c>
       <c r="B24">
-        <v>19.010000000000002</v>
-      </c>
-      <c r="C24">
-        <v>0</v>
+        <v>18.5349</v>
+      </c>
+      <c r="C24" s="3">
+        <v>7</v>
       </c>
       <c r="D24" s="2">
         <v>1.7</v>
       </c>
       <c r="E24">
-        <v>0</v>
+        <v>3.4</v>
       </c>
       <c r="F24">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G24" s="2">
         <f t="shared" si="0"/>
-        <v>73.087999999999994</v>
+        <v>84.183999999999997</v>
       </c>
       <c r="H24">
-        <v>1.08718</v>
+        <v>0.95721000000000001</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A25" t="s">
-        <v>27</v>
+        <v>36</v>
       </c>
       <c r="B25">
-        <v>19.010000000000002</v>
-      </c>
-      <c r="C25">
-        <v>0</v>
+        <v>18.5349</v>
+      </c>
+      <c r="C25" s="3">
+        <v>7</v>
       </c>
       <c r="D25" s="2">
         <v>1.7</v>
       </c>
       <c r="E25">
-        <v>0</v>
+        <v>3.4</v>
       </c>
       <c r="F25">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="G25" s="2">
         <f t="shared" si="0"/>
-        <v>84.183999999999997</v>
+        <v>96.335999999999999</v>
       </c>
       <c r="H25">
-        <v>1.07606</v>
+        <v>0.93257000000000001</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A26" t="s">
-        <v>28</v>
+        <v>37</v>
       </c>
       <c r="B26">
-        <v>19.010000000000002</v>
-      </c>
-      <c r="C26">
-        <v>0</v>
+        <v>18.5349</v>
+      </c>
+      <c r="C26" s="3">
+        <v>7</v>
       </c>
       <c r="D26" s="2">
         <v>1.7</v>
       </c>
       <c r="E26">
-        <v>0</v>
+        <v>3.4</v>
       </c>
       <c r="F26">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="G26" s="2">
         <f t="shared" si="0"/>
-        <v>96.335999999999999</v>
+        <v>109.592</v>
       </c>
       <c r="H26">
-        <v>1.0610900000000001</v>
+        <v>0.90500000000000003</v>
       </c>
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A27" t="s">
-        <v>29</v>
-      </c>
-      <c r="B27">
+      <c r="D27" s="2"/>
+      <c r="G27" s="2"/>
+    </row>
+    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>38</v>
+      </c>
+      <c r="B28">
         <v>19.010000000000002</v>
       </c>
-      <c r="C27">
-        <v>0</v>
-      </c>
-      <c r="D27" s="2">
-        <v>1.7</v>
-      </c>
-      <c r="E27">
-        <v>0</v>
-      </c>
-      <c r="F27">
-        <v>24</v>
-      </c>
-      <c r="G27" s="2">
-        <f t="shared" si="0"/>
-        <v>109.592</v>
-      </c>
-      <c r="H27">
-        <v>1.0434699999999999</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="D28" s="2"/>
-      <c r="G28" s="2"/>
+      <c r="C28" s="3">
+        <v>0</v>
+      </c>
+      <c r="D28" s="2">
+        <v>1.6</v>
+      </c>
+      <c r="E28">
+        <v>1.4</v>
+      </c>
+      <c r="F28">
+        <v>14</v>
+      </c>
+      <c r="G28" s="2">
+        <f t="shared" si="0"/>
+        <v>20.952000000000002</v>
+      </c>
+      <c r="H28">
+        <v>0.97521999999999998</v>
+      </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A29" t="s">
-        <v>30</v>
+        <v>39</v>
       </c>
       <c r="B29">
-        <v>18.53</v>
-      </c>
-      <c r="C29">
-        <v>7.1</v>
+        <v>19.010000000000002</v>
+      </c>
+      <c r="C29" s="3">
+        <v>0</v>
       </c>
       <c r="D29" s="2">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="E29">
         <v>1.4</v>
       </c>
       <c r="F29">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="G29" s="2">
         <f t="shared" si="0"/>
-        <v>12.824</v>
+        <v>26</v>
       </c>
       <c r="H29">
-        <v>0.84845999999999999</v>
+        <v>1.0164299999999999</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A30" t="s">
-        <v>31</v>
+        <v>40</v>
       </c>
       <c r="B30">
-        <v>18.53</v>
-      </c>
-      <c r="C30">
-        <v>7.1</v>
+        <v>19.010000000000002</v>
+      </c>
+      <c r="C30" s="3">
+        <v>0</v>
       </c>
       <c r="D30" s="2">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="E30">
         <v>1.4</v>
       </c>
       <c r="F30">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="G30" s="2">
         <f t="shared" si="0"/>
-        <v>16.576000000000001</v>
+        <v>31.768000000000001</v>
       </c>
       <c r="H30">
-        <v>0.91712000000000005</v>
+        <v>1.0458700000000001</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A31" t="s">
-        <v>32</v>
+        <v>41</v>
       </c>
       <c r="B31">
-        <v>18.53</v>
-      </c>
-      <c r="C31">
-        <v>7.1</v>
+        <v>19.010000000000002</v>
+      </c>
+      <c r="C31" s="3">
+        <v>0</v>
       </c>
       <c r="D31" s="2">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="E31">
         <v>1.4</v>
       </c>
       <c r="F31">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="G31" s="2">
         <f t="shared" si="0"/>
-        <v>20.952000000000002</v>
+        <v>38.304000000000002</v>
       </c>
       <c r="H31">
-        <v>0.96872000000000003</v>
+        <v>1.0630500000000001</v>
       </c>
     </row>
     <row r="32" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A32" t="s">
-        <v>33</v>
+        <v>42</v>
       </c>
       <c r="B32">
-        <v>18.53</v>
-      </c>
-      <c r="C32">
-        <v>7.1</v>
+        <v>19.010000000000002</v>
+      </c>
+      <c r="C32" s="3">
+        <v>0</v>
       </c>
       <c r="D32" s="2">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="E32">
         <v>1.4</v>
       </c>
       <c r="F32">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="G32" s="2">
         <f t="shared" si="0"/>
-        <v>26</v>
+        <v>45.655999999999999</v>
       </c>
       <c r="H32">
-        <v>1.0056700000000001</v>
+        <v>1.0724400000000001</v>
       </c>
     </row>
     <row r="33" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A33" t="s">
-        <v>34</v>
+        <v>43</v>
       </c>
       <c r="B33">
-        <v>18.53</v>
-      </c>
-      <c r="C33">
-        <v>7.1</v>
+        <v>19.010000000000002</v>
+      </c>
+      <c r="C33" s="3">
+        <v>0</v>
       </c>
       <c r="D33" s="2">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="E33">
         <v>1.4</v>
       </c>
       <c r="F33">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="G33" s="2">
         <f t="shared" si="0"/>
-        <v>31.768000000000001</v>
+        <v>53.872</v>
       </c>
       <c r="H33">
-        <v>1.03034</v>
+        <v>1.0734300000000001</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A34" t="s">
-        <v>36</v>
+        <v>44</v>
       </c>
       <c r="B34">
-        <v>18.53</v>
-      </c>
-      <c r="C34">
-        <v>7.1</v>
+        <v>19.010000000000002</v>
+      </c>
+      <c r="C34" s="3">
+        <v>0</v>
       </c>
       <c r="D34" s="2">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="E34">
         <v>1.4</v>
       </c>
       <c r="F34">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="G34" s="2">
         <f t="shared" si="0"/>
-        <v>38.304000000000002</v>
+        <v>63</v>
       </c>
       <c r="H34">
-        <v>1.04437</v>
+        <v>1.0687</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A35" t="s">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="B35">
-        <v>18.53</v>
-      </c>
-      <c r="C35">
-        <v>7.1</v>
+        <v>19.010000000000002</v>
+      </c>
+      <c r="C35" s="3">
+        <v>0</v>
       </c>
       <c r="D35" s="2">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="E35">
         <v>1.4</v>
       </c>
       <c r="F35">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="G35" s="2">
         <f t="shared" si="0"/>
-        <v>45.655999999999999</v>
+        <v>73.087999999999994</v>
       </c>
       <c r="H35">
-        <v>1.04986</v>
+        <v>1.0589999999999999</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A36" t="s">
-        <v>38</v>
+        <v>46</v>
       </c>
       <c r="B36">
-        <v>18.53</v>
-      </c>
-      <c r="C36">
-        <v>7.1</v>
+        <v>19.010000000000002</v>
+      </c>
+      <c r="C36" s="3">
+        <v>0</v>
       </c>
       <c r="D36" s="2">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="E36">
         <v>1.4</v>
       </c>
       <c r="F36">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="G36" s="2">
         <f t="shared" si="0"/>
-        <v>53.872</v>
+        <v>84.183999999999997</v>
       </c>
       <c r="H36">
-        <v>1.0482800000000001</v>
+        <v>1.04487</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A37" t="s">
-        <v>39</v>
+        <v>47</v>
       </c>
       <c r="B37">
-        <v>18.53</v>
-      </c>
-      <c r="C37">
-        <v>7.1</v>
+        <v>19.010000000000002</v>
+      </c>
+      <c r="C37" s="3">
+        <v>0</v>
       </c>
       <c r="D37" s="2">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="E37">
         <v>1.4</v>
       </c>
       <c r="F37">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="G37" s="2">
         <f t="shared" si="0"/>
-        <v>63</v>
+        <v>96.335999999999999</v>
       </c>
       <c r="H37">
-        <v>1.04074</v>
+        <v>1.0271600000000001</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A38" t="s">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="B38">
-        <v>18.53</v>
-      </c>
-      <c r="C38">
-        <v>7.1</v>
+        <v>19.010000000000002</v>
+      </c>
+      <c r="C38" s="3">
+        <v>0</v>
       </c>
       <c r="D38" s="2">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="E38">
         <v>1.4</v>
       </c>
       <c r="F38">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="G38" s="2">
         <f t="shared" si="0"/>
-        <v>73.087999999999994</v>
+        <v>109.592</v>
       </c>
       <c r="H38">
-        <v>1.02807</v>
+        <v>1.00644</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A39" t="s">
-        <v>41</v>
+        <v>65</v>
       </c>
       <c r="B39">
-        <v>18.53</v>
-      </c>
-      <c r="C39">
-        <v>7.1</v>
+        <v>19.010000000000002</v>
+      </c>
+      <c r="C39" s="3">
+        <v>0</v>
       </c>
       <c r="D39" s="2">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="E39">
         <v>1.4</v>
       </c>
       <c r="F39">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="G39" s="2">
-        <f t="shared" si="0"/>
-        <v>84.183999999999997</v>
+        <f t="shared" ref="G39:G40" si="2">((F39^3)-(5^3))/(5^3)</f>
+        <v>124</v>
       </c>
       <c r="H39">
-        <v>1.01156</v>
+        <v>0.98375000000000001</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A40" t="s">
-        <v>42</v>
+        <v>66</v>
       </c>
       <c r="B40">
-        <v>18.53</v>
-      </c>
-      <c r="C40">
-        <v>7.1</v>
+        <v>19.010000000000002</v>
+      </c>
+      <c r="C40" s="3">
+        <v>0</v>
       </c>
       <c r="D40" s="2">
-        <v>1.7</v>
+        <v>1.6</v>
       </c>
       <c r="E40">
         <v>1.4</v>
       </c>
       <c r="F40">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="G40" s="2">
-        <f t="shared" si="0"/>
-        <v>96.335999999999999</v>
+        <f t="shared" si="2"/>
+        <v>139.608</v>
       </c>
       <c r="H40">
-        <v>0.99184000000000005</v>
+        <v>0.95835999999999999</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A41" t="s">
-        <v>43</v>
-      </c>
-      <c r="B41">
-        <v>18.53</v>
-      </c>
-      <c r="C41">
-        <v>7.1</v>
-      </c>
-      <c r="D41" s="2">
+      <c r="D41" s="2"/>
+    </row>
+    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A42" t="s">
+        <v>49</v>
+      </c>
+      <c r="B42">
+        <v>19.010000000000002</v>
+      </c>
+      <c r="C42" s="3">
+        <v>0</v>
+      </c>
+      <c r="D42" s="2">
         <v>1.7</v>
       </c>
-      <c r="E41">
-        <v>1.4</v>
-      </c>
-      <c r="F41">
-        <v>24</v>
-      </c>
-      <c r="G41" s="2">
-        <f t="shared" si="0"/>
-        <v>109.592</v>
-      </c>
-      <c r="H41">
-        <v>0.96913000000000005</v>
-      </c>
-    </row>
-    <row r="42" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="D42" s="2"/>
+      <c r="E42">
+        <v>3.4</v>
+      </c>
+      <c r="F42">
+        <v>14</v>
+      </c>
+      <c r="G42" s="2">
+        <f t="shared" si="0"/>
+        <v>20.952000000000002</v>
+      </c>
+      <c r="H42">
+        <v>0.97228999999999999</v>
+      </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A43" t="s">
-        <v>46</v>
+        <v>50</v>
       </c>
       <c r="B43">
         <v>19.010000000000002</v>
       </c>
-      <c r="C43">
+      <c r="C43" s="3">
         <v>0</v>
       </c>
       <c r="D43" s="2">
         <v>1.7</v>
       </c>
       <c r="E43">
-        <v>6.6</v>
+        <v>3.4</v>
       </c>
       <c r="F43">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="G43" s="2">
         <f t="shared" si="0"/>
-        <v>12.824</v>
+        <v>26</v>
       </c>
       <c r="H43">
-        <v>0.84230000000000005</v>
+        <v>1.00552</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A44" t="s">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="B44">
         <v>19.010000000000002</v>
       </c>
-      <c r="C44">
+      <c r="C44" s="3">
         <v>0</v>
       </c>
       <c r="D44" s="2">
         <v>1.7</v>
       </c>
       <c r="E44">
-        <v>6.6</v>
+        <v>3.4</v>
       </c>
       <c r="F44">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="G44" s="2">
         <f t="shared" si="0"/>
-        <v>16.576000000000001</v>
+        <v>31.768000000000001</v>
       </c>
       <c r="H44">
-        <v>0.90561999999999998</v>
+        <v>1.02549</v>
       </c>
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A45" t="s">
-        <v>48</v>
+        <v>52</v>
       </c>
       <c r="B45">
         <v>19.010000000000002</v>
       </c>
-      <c r="C45">
+      <c r="C45" s="3">
         <v>0</v>
       </c>
       <c r="D45" s="2">
         <v>1.7</v>
       </c>
       <c r="E45">
-        <v>6.6</v>
+        <v>3.4</v>
       </c>
       <c r="F45">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="G45" s="2">
         <f t="shared" si="0"/>
-        <v>20.952000000000002</v>
+        <v>38.304000000000002</v>
       </c>
       <c r="H45">
-        <v>0.95065</v>
+        <v>1.03454</v>
       </c>
     </row>
     <row r="46" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A46" t="s">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="B46">
         <v>19.010000000000002</v>
       </c>
-      <c r="C46">
+      <c r="C46" s="3">
         <v>0</v>
       </c>
       <c r="D46" s="2">
         <v>1.7</v>
       </c>
       <c r="E46">
-        <v>6.6</v>
+        <v>3.4</v>
       </c>
       <c r="F46">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="G46" s="2">
         <f t="shared" si="0"/>
-        <v>26</v>
+        <v>45.655999999999999</v>
       </c>
       <c r="H46">
-        <v>0.97985999999999995</v>
+        <v>1.03451</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A47" t="s">
-        <v>50</v>
+        <v>54</v>
       </c>
       <c r="B47">
         <v>19.010000000000002</v>
       </c>
-      <c r="C47">
+      <c r="C47" s="3">
         <v>0</v>
       </c>
       <c r="D47" s="2">
         <v>1.7</v>
       </c>
       <c r="E47">
-        <v>6.6</v>
+        <v>3.4</v>
       </c>
       <c r="F47">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="G47" s="2">
         <f t="shared" si="0"/>
-        <v>31.768000000000001</v>
+        <v>53.872</v>
       </c>
       <c r="H47">
-        <v>0.99507000000000001</v>
+        <v>1.0269299999999999</v>
       </c>
     </row>
     <row r="48" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A48" t="s">
-        <v>51</v>
+        <v>55</v>
       </c>
       <c r="B48">
         <v>19.010000000000002</v>
       </c>
-      <c r="C48">
+      <c r="C48" s="3">
         <v>0</v>
       </c>
       <c r="D48" s="2">
         <v>1.7</v>
       </c>
       <c r="E48">
-        <v>6.6</v>
+        <v>3.4</v>
       </c>
       <c r="F48">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="G48" s="2">
         <f t="shared" si="0"/>
-        <v>38.304000000000002</v>
+        <v>63</v>
       </c>
       <c r="H48">
-        <v>0.99902000000000002</v>
+        <v>1.0133000000000001</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A49" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="B49">
         <v>19.010000000000002</v>
       </c>
-      <c r="C49">
+      <c r="C49" s="3">
         <v>0</v>
       </c>
       <c r="D49" s="2">
         <v>1.7</v>
       </c>
       <c r="E49">
-        <v>6.6</v>
+        <v>3.4</v>
       </c>
       <c r="F49">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="G49" s="2">
         <f t="shared" si="0"/>
-        <v>45.655999999999999</v>
+        <v>73.087999999999994</v>
       </c>
       <c r="H49">
-        <v>0.99387999999999999</v>
+        <v>0.99485999999999997</v>
       </c>
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A50" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="B50">
         <v>19.010000000000002</v>
       </c>
-      <c r="C50">
+      <c r="C50" s="3">
         <v>0</v>
       </c>
       <c r="D50" s="2">
         <v>1.7</v>
       </c>
       <c r="E50">
-        <v>6.6</v>
+        <v>3.4</v>
       </c>
       <c r="F50">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="G50" s="2">
         <f t="shared" si="0"/>
-        <v>53.872</v>
+        <v>84.183999999999997</v>
       </c>
       <c r="H50">
-        <v>0.98128000000000004</v>
+        <v>0.97267000000000003</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A51" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="B51">
         <v>19.010000000000002</v>
       </c>
-      <c r="C51">
+      <c r="C51" s="3">
         <v>0</v>
       </c>
       <c r="D51" s="2">
         <v>1.7</v>
       </c>
       <c r="E51">
-        <v>6.6</v>
+        <v>3.4</v>
       </c>
       <c r="F51">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="G51" s="2">
         <f t="shared" si="0"/>
-        <v>63</v>
+        <v>96.335999999999999</v>
       </c>
       <c r="H51">
-        <v>0.96287</v>
+        <v>0.94721999999999995</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A52" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="B52">
         <v>19.010000000000002</v>
       </c>
-      <c r="C52">
+      <c r="C52" s="3">
         <v>0</v>
       </c>
       <c r="D52" s="2">
         <v>1.7</v>
       </c>
       <c r="E52">
-        <v>6.6</v>
+        <v>3.4</v>
       </c>
       <c r="F52">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="G52" s="2">
         <f t="shared" si="0"/>
-        <v>73.087999999999994</v>
+        <v>109.592</v>
       </c>
       <c r="H52">
-        <v>0.93959000000000004</v>
+        <v>0.91939000000000004</v>
       </c>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A53" t="s">
-        <v>56</v>
-      </c>
-      <c r="B53">
-        <v>19.010000000000002</v>
-      </c>
-      <c r="C53">
-        <v>0</v>
-      </c>
-      <c r="D53" s="2">
-        <v>1.7</v>
-      </c>
-      <c r="E53">
-        <v>6.6</v>
-      </c>
-      <c r="F53">
-        <v>22</v>
-      </c>
-      <c r="G53" s="2">
-        <f t="shared" si="0"/>
-        <v>84.183999999999997</v>
-      </c>
-      <c r="H53">
-        <v>0.91279999999999994</v>
-      </c>
+      <c r="D53" s="2"/>
+      <c r="G53" s="2"/>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A54" t="s">
-        <v>57</v>
+        <v>4</v>
       </c>
       <c r="B54">
         <v>19.010000000000002</v>
       </c>
-      <c r="C54">
+      <c r="C54" s="3">
         <v>0</v>
       </c>
       <c r="D54" s="2">
         <v>1.7</v>
       </c>
-      <c r="E54">
-        <v>6.6</v>
+      <c r="E54" s="3">
+        <v>0</v>
       </c>
       <c r="F54">
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="G54" s="2">
         <f t="shared" si="0"/>
-        <v>96.335999999999999</v>
+        <v>20.952000000000002</v>
       </c>
       <c r="H54">
-        <v>0.88341000000000003</v>
+        <v>0.99070000000000003</v>
       </c>
     </row>
     <row r="55" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A55" t="s">
-        <v>58</v>
+        <v>5</v>
       </c>
       <c r="B55">
         <v>19.010000000000002</v>
       </c>
-      <c r="C55">
+      <c r="C55" s="3">
         <v>0</v>
       </c>
       <c r="D55" s="2">
         <v>1.7</v>
       </c>
-      <c r="E55">
+      <c r="E55" s="3">
+        <v>0</v>
+      </c>
+      <c r="F55">
+        <v>15</v>
+      </c>
+      <c r="G55" s="2">
+        <f t="shared" si="0"/>
+        <v>26</v>
+      </c>
+      <c r="H55">
+        <v>1.0325800000000001</v>
+      </c>
+    </row>
+    <row r="56" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A56" t="s">
+        <v>6</v>
+      </c>
+      <c r="B56">
+        <v>19.010000000000002</v>
+      </c>
+      <c r="C56" s="3">
+        <v>0</v>
+      </c>
+      <c r="D56" s="2">
+        <v>1.7</v>
+      </c>
+      <c r="E56" s="3">
+        <v>0</v>
+      </c>
+      <c r="F56">
+        <v>16</v>
+      </c>
+      <c r="G56" s="2">
+        <f t="shared" si="0"/>
+        <v>31.768000000000001</v>
+      </c>
+      <c r="H56">
+        <v>1.06219</v>
+      </c>
+    </row>
+    <row r="57" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A57" t="s">
+        <v>7</v>
+      </c>
+      <c r="B57">
+        <v>19.010000000000002</v>
+      </c>
+      <c r="C57" s="3">
+        <v>0</v>
+      </c>
+      <c r="D57" s="2">
+        <v>1.7</v>
+      </c>
+      <c r="E57" s="3">
+        <v>0</v>
+      </c>
+      <c r="F57">
+        <v>17</v>
+      </c>
+      <c r="G57" s="2">
+        <f t="shared" si="0"/>
+        <v>38.304000000000002</v>
+      </c>
+      <c r="H57">
+        <v>1.0817099999999999</v>
+      </c>
+    </row>
+    <row r="58" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A58" t="s">
+        <v>8</v>
+      </c>
+      <c r="B58">
+        <v>19.010000000000002</v>
+      </c>
+      <c r="C58" s="3">
+        <v>0</v>
+      </c>
+      <c r="D58" s="2">
+        <v>1.7</v>
+      </c>
+      <c r="E58" s="3">
+        <v>0</v>
+      </c>
+      <c r="F58">
+        <v>18</v>
+      </c>
+      <c r="G58" s="2">
+        <f t="shared" si="0"/>
+        <v>45.655999999999999</v>
+      </c>
+      <c r="H58">
+        <v>1.09256</v>
+      </c>
+    </row>
+    <row r="59" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A59" t="s">
+        <v>9</v>
+      </c>
+      <c r="B59">
+        <v>19.010000000000002</v>
+      </c>
+      <c r="C59" s="3">
+        <v>0</v>
+      </c>
+      <c r="D59" s="2">
+        <v>1.7</v>
+      </c>
+      <c r="E59" s="3">
+        <v>0</v>
+      </c>
+      <c r="F59">
+        <v>19</v>
+      </c>
+      <c r="G59" s="2">
+        <f t="shared" si="0"/>
+        <v>53.872</v>
+      </c>
+      <c r="H59">
+        <v>1.09642</v>
+      </c>
+    </row>
+    <row r="60" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A60" t="s">
+        <v>10</v>
+      </c>
+      <c r="B60">
+        <v>19.010000000000002</v>
+      </c>
+      <c r="C60" s="3">
+        <v>0</v>
+      </c>
+      <c r="D60" s="2">
+        <v>1.7</v>
+      </c>
+      <c r="E60" s="3">
+        <v>0</v>
+      </c>
+      <c r="F60">
+        <v>20</v>
+      </c>
+      <c r="G60" s="2">
+        <f t="shared" si="0"/>
+        <v>63</v>
+      </c>
+      <c r="H60">
+        <v>1.0943400000000001</v>
+      </c>
+    </row>
+    <row r="61" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A61" t="s">
+        <v>11</v>
+      </c>
+      <c r="B61">
+        <v>19.010000000000002</v>
+      </c>
+      <c r="C61" s="3">
+        <v>0</v>
+      </c>
+      <c r="D61" s="2">
+        <v>1.7</v>
+      </c>
+      <c r="E61" s="3">
+        <v>0</v>
+      </c>
+      <c r="F61">
+        <v>21</v>
+      </c>
+      <c r="G61" s="2">
+        <f t="shared" si="0"/>
+        <v>73.087999999999994</v>
+      </c>
+      <c r="H61">
+        <v>1.08718</v>
+      </c>
+    </row>
+    <row r="62" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A62" t="s">
+        <v>12</v>
+      </c>
+      <c r="B62">
+        <v>19.010000000000002</v>
+      </c>
+      <c r="C62" s="3">
+        <v>0</v>
+      </c>
+      <c r="D62" s="2">
+        <v>1.7</v>
+      </c>
+      <c r="E62" s="3">
+        <v>0</v>
+      </c>
+      <c r="F62">
+        <v>22</v>
+      </c>
+      <c r="G62" s="2">
+        <f t="shared" si="0"/>
+        <v>84.183999999999997</v>
+      </c>
+      <c r="H62">
+        <v>1.07606</v>
+      </c>
+    </row>
+    <row r="63" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A63" t="s">
+        <v>13</v>
+      </c>
+      <c r="B63">
+        <v>19.010000000000002</v>
+      </c>
+      <c r="C63" s="3">
+        <v>0</v>
+      </c>
+      <c r="D63" s="2">
+        <v>1.7</v>
+      </c>
+      <c r="E63" s="3">
+        <v>0</v>
+      </c>
+      <c r="F63">
+        <v>23</v>
+      </c>
+      <c r="G63" s="2">
+        <f t="shared" si="0"/>
+        <v>96.335999999999999</v>
+      </c>
+      <c r="H63">
+        <v>1.0610900000000001</v>
+      </c>
+    </row>
+    <row r="64" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A64" t="s">
+        <v>14</v>
+      </c>
+      <c r="B64">
+        <v>19.010000000000002</v>
+      </c>
+      <c r="C64" s="3">
+        <v>0</v>
+      </c>
+      <c r="D64" s="2">
+        <v>1.7</v>
+      </c>
+      <c r="E64" s="3">
+        <v>0</v>
+      </c>
+      <c r="F64">
+        <v>24</v>
+      </c>
+      <c r="G64" s="2">
+        <f t="shared" si="0"/>
+        <v>109.592</v>
+      </c>
+      <c r="H64">
+        <v>1.0434699999999999</v>
+      </c>
+    </row>
+    <row r="65" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A65" t="s">
+        <v>63</v>
+      </c>
+      <c r="B65">
+        <v>19.010000000000002</v>
+      </c>
+      <c r="C65" s="3">
+        <v>0</v>
+      </c>
+      <c r="D65" s="2">
+        <v>1.7</v>
+      </c>
+      <c r="E65" s="3">
+        <v>0</v>
+      </c>
+      <c r="F65">
+        <v>25</v>
+      </c>
+      <c r="G65" s="2">
+        <f t="shared" ref="G65:G66" si="3">((F65^3)-(5^3))/(5^3)</f>
+        <v>124</v>
+      </c>
+      <c r="H65">
+        <v>1.02311</v>
+      </c>
+    </row>
+    <row r="66" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A66" t="s">
+        <v>64</v>
+      </c>
+      <c r="B66">
+        <v>19.010000000000002</v>
+      </c>
+      <c r="C66" s="3">
+        <v>0</v>
+      </c>
+      <c r="D66" s="2">
+        <v>1.7</v>
+      </c>
+      <c r="E66" s="3">
+        <v>0</v>
+      </c>
+      <c r="F66">
+        <v>26</v>
+      </c>
+      <c r="G66" s="2">
+        <f t="shared" si="3"/>
+        <v>139.608</v>
+      </c>
+      <c r="H66">
+        <v>1.00098</v>
+      </c>
+    </row>
+    <row r="68" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A68" t="s">
+        <v>67</v>
+      </c>
+      <c r="B68">
+        <v>18.5349</v>
+      </c>
+      <c r="C68" s="3">
+        <v>7</v>
+      </c>
+      <c r="D68" s="2">
+        <v>1.6</v>
+      </c>
+      <c r="E68">
         <v>6.6</v>
       </c>
-      <c r="F55">
-        <v>24</v>
-      </c>
-      <c r="G55" s="2">
-        <f t="shared" si="0"/>
-        <v>109.592</v>
-      </c>
-      <c r="H55">
-        <v>0.85238000000000003</v>
+      <c r="F68">
+        <v>12</v>
+      </c>
+      <c r="G68" s="2">
+        <f>((F68^3)-(5^3))/(5^3)</f>
+        <v>12.824</v>
+      </c>
+      <c r="H68">
+        <v>0.83423999999999998</v>
+      </c>
+    </row>
+    <row r="69" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A69" t="s">
+        <v>68</v>
+      </c>
+      <c r="B69">
+        <v>18.5349</v>
+      </c>
+      <c r="C69" s="3">
+        <v>7</v>
+      </c>
+      <c r="D69" s="2">
+        <v>1.6</v>
+      </c>
+      <c r="E69">
+        <v>6.6</v>
+      </c>
+      <c r="F69">
+        <v>13</v>
+      </c>
+      <c r="G69" s="2">
+        <f t="shared" ref="G69:G78" si="4">((F69^3)-(5^3))/(5^3)</f>
+        <v>16.576000000000001</v>
+      </c>
+      <c r="H69">
+        <v>0.89614000000000005</v>
+      </c>
+    </row>
+    <row r="70" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A70" t="s">
+        <v>69</v>
+      </c>
+      <c r="B70">
+        <v>18.5349</v>
+      </c>
+      <c r="C70" s="3">
+        <v>7</v>
+      </c>
+      <c r="D70" s="2">
+        <v>1.6</v>
+      </c>
+      <c r="E70">
+        <v>6.6</v>
+      </c>
+      <c r="F70">
+        <v>14</v>
+      </c>
+      <c r="G70" s="2">
+        <f t="shared" si="4"/>
+        <v>20.952000000000002</v>
+      </c>
+      <c r="H70">
+        <v>0.93979000000000001</v>
+      </c>
+    </row>
+    <row r="71" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A71" t="s">
+        <v>70</v>
+      </c>
+      <c r="B71">
+        <v>18.5349</v>
+      </c>
+      <c r="C71" s="3">
+        <v>7</v>
+      </c>
+      <c r="D71" s="2">
+        <v>1.6</v>
+      </c>
+      <c r="E71">
+        <v>6.6</v>
+      </c>
+      <c r="F71">
+        <v>15</v>
+      </c>
+      <c r="G71" s="2">
+        <f t="shared" si="4"/>
+        <v>26</v>
+      </c>
+      <c r="H71">
+        <v>0.96750000000000003</v>
+      </c>
+    </row>
+    <row r="72" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A72" t="s">
+        <v>71</v>
+      </c>
+      <c r="B72">
+        <v>18.5349</v>
+      </c>
+      <c r="C72" s="3">
+        <v>7</v>
+      </c>
+      <c r="D72" s="2">
+        <v>1.6</v>
+      </c>
+      <c r="E72">
+        <v>6.6</v>
+      </c>
+      <c r="F72">
+        <v>16</v>
+      </c>
+      <c r="G72" s="2">
+        <f t="shared" si="4"/>
+        <v>31.768000000000001</v>
+      </c>
+      <c r="H72">
+        <v>0.98211000000000004</v>
+      </c>
+    </row>
+    <row r="73" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A73" t="s">
+        <v>72</v>
+      </c>
+      <c r="B73">
+        <v>18.5349</v>
+      </c>
+      <c r="C73" s="3">
+        <v>7</v>
+      </c>
+      <c r="D73" s="2">
+        <v>1.6</v>
+      </c>
+      <c r="E73">
+        <v>6.6</v>
+      </c>
+      <c r="F73">
+        <v>17</v>
+      </c>
+      <c r="G73" s="2">
+        <f t="shared" si="4"/>
+        <v>38.304000000000002</v>
+      </c>
+      <c r="H73">
+        <v>0.98540000000000005</v>
+      </c>
+    </row>
+    <row r="74" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A74" t="s">
+        <v>73</v>
+      </c>
+      <c r="B74">
+        <v>18.5349</v>
+      </c>
+      <c r="C74" s="3">
+        <v>7</v>
+      </c>
+      <c r="D74" s="2">
+        <v>1.6</v>
+      </c>
+      <c r="E74">
+        <v>6.6</v>
+      </c>
+      <c r="F74">
+        <v>18</v>
+      </c>
+      <c r="G74" s="2">
+        <f t="shared" si="4"/>
+        <v>45.655999999999999</v>
+      </c>
+      <c r="H74">
+        <v>0.98006000000000004</v>
+      </c>
+    </row>
+    <row r="75" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A75" t="s">
+        <v>74</v>
+      </c>
+      <c r="B75">
+        <v>18.5349</v>
+      </c>
+      <c r="C75" s="3">
+        <v>7</v>
+      </c>
+      <c r="D75" s="2">
+        <v>1.6</v>
+      </c>
+      <c r="E75">
+        <v>6.6</v>
+      </c>
+      <c r="F75">
+        <v>19</v>
+      </c>
+      <c r="G75" s="2">
+        <f t="shared" si="4"/>
+        <v>53.872</v>
+      </c>
+      <c r="H75">
+        <v>0.96731</v>
+      </c>
+    </row>
+    <row r="76" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A76" t="s">
+        <v>75</v>
+      </c>
+      <c r="B76">
+        <v>18.5349</v>
+      </c>
+      <c r="C76" s="3">
+        <v>7</v>
+      </c>
+      <c r="D76" s="2">
+        <v>1.6</v>
+      </c>
+      <c r="E76">
+        <v>6.6</v>
+      </c>
+      <c r="F76">
+        <v>20</v>
+      </c>
+      <c r="G76" s="2">
+        <f t="shared" si="4"/>
+        <v>63</v>
+      </c>
+      <c r="H76">
+        <v>0.94891999999999999</v>
+      </c>
+    </row>
+    <row r="77" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A77" t="s">
+        <v>76</v>
+      </c>
+      <c r="B77">
+        <v>18.5349</v>
+      </c>
+      <c r="C77" s="3">
+        <v>7</v>
+      </c>
+      <c r="D77" s="2">
+        <v>1.6</v>
+      </c>
+      <c r="E77">
+        <v>6.6</v>
+      </c>
+      <c r="F77">
+        <v>21</v>
+      </c>
+      <c r="G77" s="2">
+        <f t="shared" si="4"/>
+        <v>73.087999999999994</v>
+      </c>
+      <c r="H77">
+        <v>0.92556000000000005</v>
+      </c>
+    </row>
+    <row r="78" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A78" t="s">
+        <v>77</v>
+      </c>
+      <c r="B78">
+        <v>18.5349</v>
+      </c>
+      <c r="C78" s="3">
+        <v>7</v>
+      </c>
+      <c r="D78" s="2">
+        <v>1.6</v>
+      </c>
+      <c r="E78">
+        <v>6.6</v>
+      </c>
+      <c r="F78">
+        <v>22</v>
+      </c>
+      <c r="G78" s="2">
+        <f t="shared" si="4"/>
+        <v>84.183999999999997</v>
+      </c>
+      <c r="H78">
+        <v>0.89922999999999997</v>
       </c>
     </row>
   </sheetData>

</xml_diff>